<commit_message>
Tab 10: XLDD 1 lan thieu data -> tu dong Dat 2d (chot 25/10)
</commit_message>
<xml_diff>
--- a/VUOT-TROI-2026.xlsx
+++ b/VUOT-TROI-2026.xlsx
@@ -3075,7 +3075,7 @@
         <v>20</v>
       </c>
       <c r="H6" s="17" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I6" s="17" t="n">
         <v>20</v>
@@ -3090,7 +3090,7 @@
         <v>4</v>
       </c>
       <c r="M6" s="18" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="N6" s="19" t="inlineStr">
         <is>
@@ -3652,9 +3652,15 @@
       <c r="HW6" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="HX6" s="22" t="n"/>
-      <c r="HY6" s="22" t="n"/>
-      <c r="HZ6" s="21" t="n"/>
+      <c r="HX6" s="22" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY6" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ6" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="IA6" s="20" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -3688,7 +3694,7 @@
         <v>2</v>
       </c>
       <c r="IM6" s="24" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="IN6" s="21" t="n">
         <v>1</v>
@@ -3722,7 +3728,9 @@
       </c>
       <c r="IX6" s="22" t="n"/>
       <c r="IY6" s="22" t="n"/>
-      <c r="IZ6" s="21" t="n"/>
+      <c r="IZ6" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="JA6" s="20" t="n">
         <v>9.9</v>
       </c>
@@ -3756,7 +3764,7 @@
         <v>2</v>
       </c>
       <c r="JM6" s="24" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="JN6" s="21" t="n">
         <v>1</v>
@@ -3788,7 +3796,7 @@
         <v>20</v>
       </c>
       <c r="H7" s="17" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I7" s="17" t="n">
         <v>20</v>
@@ -3803,7 +3811,7 @@
         <v>4</v>
       </c>
       <c r="M7" s="18" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="N7" s="19" t="inlineStr">
         <is>
@@ -4365,9 +4373,15 @@
       <c r="HW7" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="HX7" s="30" t="n"/>
-      <c r="HY7" s="30" t="n"/>
-      <c r="HZ7" s="29" t="n"/>
+      <c r="HX7" s="30" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY7" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ7" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="IA7" s="28" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -4401,7 +4415,7 @@
         <v>2</v>
       </c>
       <c r="IM7" s="32" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="IN7" s="29" t="n">
         <v>1</v>
@@ -4435,7 +4449,9 @@
       </c>
       <c r="IX7" s="30" t="n"/>
       <c r="IY7" s="30" t="n"/>
-      <c r="IZ7" s="29" t="n"/>
+      <c r="IZ7" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="JA7" s="28" t="n">
         <v>9.9</v>
       </c>
@@ -4469,7 +4485,7 @@
         <v>2</v>
       </c>
       <c r="JM7" s="32" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="JN7" s="29" t="n">
         <v>1</v>
@@ -4501,7 +4517,7 @@
         <v>20</v>
       </c>
       <c r="H8" s="17" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I8" s="17" t="n">
         <v>20</v>
@@ -4516,7 +4532,7 @@
         <v>2</v>
       </c>
       <c r="M8" s="18" t="n">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="N8" s="19" t="inlineStr">
         <is>
@@ -5078,9 +5094,15 @@
       <c r="HW8" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="HX8" s="22" t="n"/>
-      <c r="HY8" s="22" t="n"/>
-      <c r="HZ8" s="21" t="n"/>
+      <c r="HX8" s="22" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY8" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ8" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="IA8" s="20" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -5114,7 +5136,7 @@
         <v>0</v>
       </c>
       <c r="IM8" s="24" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="IN8" s="21" t="n">
         <v>1</v>
@@ -5148,7 +5170,9 @@
       </c>
       <c r="IX8" s="22" t="n"/>
       <c r="IY8" s="22" t="n"/>
-      <c r="IZ8" s="21" t="n"/>
+      <c r="IZ8" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="JA8" s="20" t="n">
         <v>9.9</v>
       </c>
@@ -5182,7 +5206,7 @@
         <v>2</v>
       </c>
       <c r="JM8" s="24" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="JN8" s="21" t="n">
         <v>1</v>
@@ -5214,7 +5238,7 @@
         <v>20</v>
       </c>
       <c r="H9" s="17" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I9" s="17" t="n">
         <v>20</v>
@@ -5229,7 +5253,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="18" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="N9" s="19" t="inlineStr">
         <is>
@@ -5791,9 +5815,15 @@
       <c r="HW9" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="HX9" s="30" t="n"/>
-      <c r="HY9" s="30" t="n"/>
-      <c r="HZ9" s="29" t="n"/>
+      <c r="HX9" s="30" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY9" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ9" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="IA9" s="28" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -5827,7 +5857,7 @@
         <v>0</v>
       </c>
       <c r="IM9" s="32" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="IN9" s="29" t="n">
         <v>4</v>
@@ -5861,7 +5891,9 @@
       </c>
       <c r="IX9" s="30" t="n"/>
       <c r="IY9" s="30" t="n"/>
-      <c r="IZ9" s="29" t="n"/>
+      <c r="IZ9" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="JA9" s="28" t="n">
         <v>9.9</v>
       </c>
@@ -5893,7 +5925,7 @@
         <v>0</v>
       </c>
       <c r="JM9" s="32" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="JN9" s="29" t="n">
         <v>4</v>
@@ -5925,7 +5957,7 @@
         <v>20</v>
       </c>
       <c r="H10" s="17" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I10" s="17" t="n">
         <v>20</v>
@@ -5940,7 +5972,7 @@
         <v>2</v>
       </c>
       <c r="M10" s="18" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="N10" s="19" t="inlineStr">
         <is>
@@ -6502,9 +6534,15 @@
       <c r="HW10" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="HX10" s="22" t="n"/>
-      <c r="HY10" s="22" t="n"/>
-      <c r="HZ10" s="21" t="n"/>
+      <c r="HX10" s="22" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY10" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ10" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="IA10" s="20" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -6538,7 +6576,7 @@
         <v>0</v>
       </c>
       <c r="IM10" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="IN10" s="21" t="n">
         <v>6</v>
@@ -6572,7 +6610,9 @@
       </c>
       <c r="IX10" s="22" t="n"/>
       <c r="IY10" s="22" t="n"/>
-      <c r="IZ10" s="21" t="n"/>
+      <c r="IZ10" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="JA10" s="20" t="n">
         <v>9.9</v>
       </c>
@@ -6606,7 +6646,7 @@
         <v>2</v>
       </c>
       <c r="JM10" s="24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="JN10" s="21" t="n">
         <v>5</v>
@@ -6638,7 +6678,7 @@
         <v>20</v>
       </c>
       <c r="H11" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I11" s="17" t="n">
         <v>20</v>
@@ -6653,7 +6693,7 @@
         <v>2</v>
       </c>
       <c r="M11" s="18" t="n">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="N11" s="19" t="inlineStr">
         <is>
@@ -7215,9 +7255,15 @@
       <c r="HW11" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="HX11" s="30" t="n"/>
-      <c r="HY11" s="30" t="n"/>
-      <c r="HZ11" s="29" t="n"/>
+      <c r="HX11" s="30" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY11" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ11" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="IA11" s="28" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -7251,7 +7297,7 @@
         <v>2</v>
       </c>
       <c r="IM11" s="32" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="IN11" s="29" t="n">
         <v>5</v>
@@ -7285,7 +7331,9 @@
       </c>
       <c r="IX11" s="30" t="n"/>
       <c r="IY11" s="30" t="n"/>
-      <c r="IZ11" s="29" t="n"/>
+      <c r="IZ11" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="JA11" s="28" t="n">
         <v>9.9</v>
       </c>
@@ -7317,7 +7365,7 @@
         <v>0</v>
       </c>
       <c r="JM11" s="32" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="JN11" s="29" t="n">
         <v>6</v>
@@ -7349,7 +7397,7 @@
         <v>20</v>
       </c>
       <c r="H12" s="17" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I12" s="17" t="n">
         <v>18</v>
@@ -7364,7 +7412,7 @@
         <v>4</v>
       </c>
       <c r="M12" s="18" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="N12" s="19" t="inlineStr">
         <is>
@@ -7926,9 +7974,15 @@
       <c r="HW12" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="HX12" s="22" t="n"/>
-      <c r="HY12" s="22" t="n"/>
-      <c r="HZ12" s="21" t="n"/>
+      <c r="HX12" s="22" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY12" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ12" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="IA12" s="20" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -7962,7 +8016,7 @@
         <v>2</v>
       </c>
       <c r="IM12" s="24" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="IN12" s="21" t="n">
         <v>3</v>
@@ -7996,7 +8050,9 @@
       </c>
       <c r="IX12" s="22" t="n"/>
       <c r="IY12" s="22" t="n"/>
-      <c r="IZ12" s="21" t="n"/>
+      <c r="IZ12" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="JA12" s="20" t="n">
         <v>9.9</v>
       </c>
@@ -8030,7 +8086,7 @@
         <v>2</v>
       </c>
       <c r="JM12" s="24" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="JN12" s="21" t="n">
         <v>5</v>
@@ -8062,7 +8118,7 @@
         <v>20</v>
       </c>
       <c r="H13" s="17" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I13" s="17" t="n">
         <v>20</v>
@@ -8077,7 +8133,7 @@
         <v>4</v>
       </c>
       <c r="M13" s="18" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="N13" s="19" t="inlineStr">
         <is>
@@ -8639,9 +8695,15 @@
       <c r="HW13" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="HX13" s="30" t="n"/>
-      <c r="HY13" s="30" t="n"/>
-      <c r="HZ13" s="29" t="n"/>
+      <c r="HX13" s="30" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY13" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ13" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="IA13" s="28" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -8675,7 +8737,7 @@
         <v>2</v>
       </c>
       <c r="IM13" s="32" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="IN13" s="29" t="n">
         <v>1</v>
@@ -8709,7 +8771,9 @@
       </c>
       <c r="IX13" s="30" t="n"/>
       <c r="IY13" s="30" t="n"/>
-      <c r="IZ13" s="29" t="n"/>
+      <c r="IZ13" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="JA13" s="28" t="n">
         <v>9.9</v>
       </c>
@@ -8743,7 +8807,7 @@
         <v>2</v>
       </c>
       <c r="JM13" s="32" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="JN13" s="29" t="n">
         <v>1</v>
@@ -8775,7 +8839,7 @@
         <v>20</v>
       </c>
       <c r="H14" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I14" s="17" t="n">
         <v>20</v>
@@ -8790,7 +8854,7 @@
         <v>2</v>
       </c>
       <c r="M14" s="18" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="N14" s="19" t="inlineStr">
         <is>
@@ -9352,9 +9416,15 @@
       <c r="HW14" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="HX14" s="22" t="n"/>
-      <c r="HY14" s="22" t="n"/>
-      <c r="HZ14" s="21" t="n"/>
+      <c r="HX14" s="22" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY14" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ14" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="IA14" s="20" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -9388,7 +9458,7 @@
         <v>2</v>
       </c>
       <c r="IM14" s="24" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="IN14" s="21" t="n">
         <v>5</v>
@@ -9422,7 +9492,9 @@
       </c>
       <c r="IX14" s="22" t="n"/>
       <c r="IY14" s="22" t="n"/>
-      <c r="IZ14" s="21" t="n"/>
+      <c r="IZ14" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="JA14" s="20" t="n">
         <v>9.9</v>
       </c>
@@ -9454,7 +9526,7 @@
         <v>0</v>
       </c>
       <c r="JM14" s="24" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="JN14" s="21" t="n">
         <v>3</v>
@@ -9486,7 +9558,7 @@
         <v>20</v>
       </c>
       <c r="H15" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I15" s="17" t="n">
         <v>20</v>
@@ -9501,7 +9573,7 @@
         <v>2</v>
       </c>
       <c r="M15" s="18" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="N15" s="19" t="inlineStr">
         <is>
@@ -10063,9 +10135,15 @@
       <c r="HW15" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="HX15" s="30" t="n"/>
-      <c r="HY15" s="30" t="n"/>
-      <c r="HZ15" s="29" t="n"/>
+      <c r="HX15" s="30" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY15" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ15" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="IA15" s="28" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -10097,7 +10175,7 @@
         <v>0</v>
       </c>
       <c r="IM15" s="32" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="IN15" s="29" t="n">
         <v>3</v>
@@ -10131,7 +10209,9 @@
       </c>
       <c r="IX15" s="30" t="n"/>
       <c r="IY15" s="30" t="n"/>
-      <c r="IZ15" s="29" t="n"/>
+      <c r="IZ15" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="JA15" s="28" t="n">
         <v>9.9</v>
       </c>
@@ -10165,7 +10245,7 @@
         <v>2</v>
       </c>
       <c r="JM15" s="32" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="JN15" s="29" t="n">
         <v>1</v>
@@ -10197,7 +10277,7 @@
         <v>20</v>
       </c>
       <c r="H16" s="17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="I16" s="17" t="n">
         <v>20</v>
@@ -10212,7 +10292,7 @@
         <v>2</v>
       </c>
       <c r="M16" s="18" t="n">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
@@ -10774,9 +10854,15 @@
       <c r="HW16" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="HX16" s="22" t="n"/>
-      <c r="HY16" s="22" t="n"/>
-      <c r="HZ16" s="21" t="n"/>
+      <c r="HX16" s="22" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY16" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ16" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="IA16" s="20" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -10810,7 +10896,7 @@
         <v>2</v>
       </c>
       <c r="IM16" s="24" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="IN16" s="21" t="n">
         <v>1</v>
@@ -10844,7 +10930,9 @@
       </c>
       <c r="IX16" s="22" t="n"/>
       <c r="IY16" s="22" t="n"/>
-      <c r="IZ16" s="21" t="n"/>
+      <c r="IZ16" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="JA16" s="20" t="n">
         <v>9.9</v>
       </c>
@@ -10876,7 +10964,7 @@
         <v>0</v>
       </c>
       <c r="JM16" s="24" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="JN16" s="21" t="n">
         <v>3</v>
@@ -10908,7 +10996,7 @@
         <v>20</v>
       </c>
       <c r="H17" s="17" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I17" s="17" t="n">
         <v>20</v>
@@ -10923,7 +11011,7 @@
         <v>2</v>
       </c>
       <c r="M17" s="18" t="n">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
@@ -11485,9 +11573,15 @@
       <c r="HW17" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="HX17" s="30" t="n"/>
-      <c r="HY17" s="30" t="n"/>
-      <c r="HZ17" s="29" t="n"/>
+      <c r="HX17" s="30" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY17" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ17" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="IA17" s="28" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -11521,7 +11615,7 @@
         <v>2</v>
       </c>
       <c r="IM17" s="32" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="IN17" s="29" t="n">
         <v>7</v>
@@ -11555,7 +11649,9 @@
       </c>
       <c r="IX17" s="30" t="n"/>
       <c r="IY17" s="30" t="n"/>
-      <c r="IZ17" s="29" t="n"/>
+      <c r="IZ17" s="29" t="n">
+        <v>2</v>
+      </c>
       <c r="JA17" s="28" t="n">
         <v>9.9</v>
       </c>
@@ -11587,7 +11683,7 @@
         <v>0</v>
       </c>
       <c r="JM17" s="32" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="JN17" s="29" t="n">
         <v>7</v>
@@ -11619,7 +11715,7 @@
         <v>20</v>
       </c>
       <c r="H18" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="I18" s="17" t="n">
         <v>20</v>
@@ -11634,7 +11730,7 @@
         <v>2</v>
       </c>
       <c r="M18" s="18" t="n">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="N18" s="19" t="inlineStr">
         <is>
@@ -12196,9 +12292,15 @@
       <c r="HW18" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="HX18" s="22" t="n"/>
-      <c r="HY18" s="22" t="n"/>
-      <c r="HZ18" s="21" t="n"/>
+      <c r="HX18" s="22" t="n">
+        <v>0.9998</v>
+      </c>
+      <c r="HY18" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="HZ18" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="IA18" s="20" t="n">
         <v>9.859999999999999</v>
       </c>
@@ -12230,7 +12332,7 @@
         <v>0</v>
       </c>
       <c r="IM18" s="24" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="IN18" s="21" t="n">
         <v>6</v>
@@ -12264,7 +12366,9 @@
       </c>
       <c r="IX18" s="22" t="n"/>
       <c r="IY18" s="22" t="n"/>
-      <c r="IZ18" s="21" t="n"/>
+      <c r="IZ18" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="JA18" s="20" t="n">
         <v>9.9</v>
       </c>
@@ -12298,7 +12402,7 @@
         <v>2</v>
       </c>
       <c r="JM18" s="24" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="JN18" s="21" t="n">
         <v>5</v>
@@ -70088,7 +70192,7 @@
       </c>
       <c r="C4" s="51" t="inlineStr">
         <is>
-          <t>Lũy kế T1–T10/2026 — Tháng 10 chốt đủ tháng (31/10/2026).</t>
+          <t>Lũy kế T1–T10/2026 — Tháng 10 chốt data tới 25/10/2026 (chưa hết tháng).</t>
         </is>
       </c>
     </row>

</xml_diff>